<commit_message>
update scripts following final simulations
</commit_message>
<xml_diff>
--- a/Tools/LULC_class_aggregation.xlsx
+++ b/Tools/LULC_class_aggregation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\publication\production_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH_HPC\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DC1AC9-0A8C-4D5F-848C-6D8813EAD141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7150C2-BB2F-41DF-8002-A52E3EBAB9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="241">
   <si>
     <t>Industrie- und Gewerbegebäude</t>
   </si>
@@ -748,15 +748,6 @@
   </si>
   <si>
     <t>Shrubland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urban/amenities </t>
-  </si>
-  <si>
-    <t>Overgrown/shrubland</t>
-  </si>
-  <si>
-    <t>Aggregated_class_short</t>
   </si>
 </sst>
 </file>
@@ -872,7 +863,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -904,9 +895,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -927,9 +915,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -967,7 +955,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1073,7 +1061,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1215,7 +1203,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1223,14 +1211,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C81117-CCD0-4C70-9A30-E4F720811826}">
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultColWidth="39.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" style="5" customWidth="1"/>
     <col min="2" max="16384" width="39.7109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
@@ -1250,13 +1238,10 @@
         <v>219</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="H1" s="5" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1275,14 +1260,11 @@
       <c r="F2" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1301,14 +1283,11 @@
       <c r="F3" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1327,14 +1306,11 @@
       <c r="F4" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1353,14 +1329,11 @@
       <c r="F5" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H5" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1379,14 +1352,11 @@
       <c r="F6" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1405,14 +1375,11 @@
       <c r="F7" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1431,14 +1398,11 @@
       <c r="F8" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1457,14 +1421,11 @@
       <c r="F9" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1483,14 +1444,11 @@
       <c r="F10" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1509,14 +1467,11 @@
       <c r="F11" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1535,14 +1490,11 @@
       <c r="F12" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G12" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H12" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1561,14 +1513,11 @@
       <c r="F13" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1587,14 +1536,11 @@
       <c r="F14" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H14" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1613,14 +1559,11 @@
       <c r="F15" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G15" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H15" s="5" t="s">
+      <c r="G15" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1642,11 +1585,8 @@
       <c r="G16" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H16" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1668,11 +1608,8 @@
       <c r="G17" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H17" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1694,11 +1631,8 @@
       <c r="G18" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H18" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1720,11 +1654,8 @@
       <c r="G19" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H19" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1743,14 +1674,11 @@
       <c r="F20" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G20" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H20" s="5" t="s">
+      <c r="G20" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1772,11 +1700,8 @@
       <c r="G21" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H21" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1798,11 +1723,8 @@
       <c r="G22" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H22" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1824,11 +1746,8 @@
       <c r="G23" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H23" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1850,11 +1769,8 @@
       <c r="G24" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H24" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1876,11 +1792,8 @@
       <c r="G25" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H25" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1902,11 +1815,8 @@
       <c r="G26" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H26" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1928,11 +1838,8 @@
       <c r="G27" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H27" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1954,11 +1861,8 @@
       <c r="G28" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H28" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1980,11 +1884,8 @@
       <c r="G29" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H29" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2003,14 +1904,11 @@
       <c r="F30" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G30" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H30" s="5" t="s">
+      <c r="G30" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2029,14 +1927,11 @@
       <c r="F31" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H31" s="5" t="s">
+      <c r="G31" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2055,14 +1950,11 @@
       <c r="F32" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H32" s="5" t="s">
+      <c r="G32" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2081,14 +1973,11 @@
       <c r="F33" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G33" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H33" s="5" t="s">
+      <c r="G33" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2107,14 +1996,11 @@
       <c r="F34" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G34" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H34" s="5" t="s">
+      <c r="G34" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2133,14 +2019,11 @@
       <c r="F35" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G35" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H35" s="5" t="s">
+      <c r="G35" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2159,14 +2042,11 @@
       <c r="F36" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G36" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H36" s="5" t="s">
+      <c r="G36" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2185,14 +2065,11 @@
       <c r="F37" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G37" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="H37" s="5" t="s">
+      <c r="G37" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2211,14 +2088,11 @@
       <c r="F38" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G38" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H38" s="5" t="s">
+      <c r="G38" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2237,14 +2111,11 @@
       <c r="F39" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G39" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H39" s="5" t="s">
+      <c r="G39" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2263,14 +2134,11 @@
       <c r="F40" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G40" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H40" s="5" t="s">
+      <c r="G40" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2289,14 +2157,11 @@
       <c r="F41" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G41" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H41" s="5" t="s">
+      <c r="G41" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2315,14 +2180,11 @@
       <c r="F42" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="G42" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="H42" s="5" t="s">
+      <c r="G42" s="5" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2341,14 +2203,11 @@
       <c r="F43" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G43" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H43" s="5" t="s">
+      <c r="G43" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2367,14 +2226,11 @@
       <c r="F44" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H44" s="5" t="s">
+      <c r="G44" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2393,14 +2249,11 @@
       <c r="F45" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G45" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H45" s="5" t="s">
+      <c r="G45" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2419,14 +2272,11 @@
       <c r="F46" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G46" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H46" s="5" t="s">
+      <c r="G46" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2445,14 +2295,11 @@
       <c r="F47" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G47" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H47" s="5" t="s">
+      <c r="G47" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2471,14 +2318,11 @@
       <c r="F48" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G48" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H48" s="5" t="s">
+      <c r="G48" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2497,14 +2341,11 @@
       <c r="F49" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G49" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H49" s="5" t="s">
+      <c r="G49" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2523,14 +2364,11 @@
       <c r="F50" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G50" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H50" s="5" t="s">
+      <c r="G50" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2549,14 +2387,11 @@
       <c r="F51" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G51" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H51" s="5" t="s">
+      <c r="G51" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2575,14 +2410,11 @@
       <c r="F52" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G52" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H52" s="5" t="s">
+      <c r="G52" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2601,14 +2433,11 @@
       <c r="F53" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G53" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H53" s="5" t="s">
+      <c r="G53" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2627,14 +2456,11 @@
       <c r="F54" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G54" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H54" s="5" t="s">
+      <c r="G54" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2653,14 +2479,11 @@
       <c r="F55" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G55" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H55" s="5" t="s">
+      <c r="G55" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2679,14 +2502,11 @@
       <c r="F56" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G56" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H56" s="5" t="s">
+      <c r="G56" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2705,14 +2525,11 @@
       <c r="F57" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G57" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H57" s="5" t="s">
+      <c r="G57" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2731,14 +2548,11 @@
       <c r="F58" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G58" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H58" s="5" t="s">
+      <c r="G58" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2757,14 +2571,11 @@
       <c r="F59" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G59" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H59" s="5" t="s">
+      <c r="G59" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2783,14 +2594,11 @@
       <c r="F60" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G60" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H60" s="5" t="s">
+      <c r="G60" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2809,14 +2617,11 @@
       <c r="F61" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G61" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H61" s="5" t="s">
+      <c r="G61" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2838,11 +2643,8 @@
       <c r="G62" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H62" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2864,11 +2666,8 @@
       <c r="G63" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H63" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2890,11 +2689,8 @@
       <c r="G64" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H64" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2913,14 +2709,11 @@
       <c r="F65" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="G65" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="H65" s="5" t="s">
+      <c r="G65" s="5" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2939,14 +2732,11 @@
       <c r="F66" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="G66" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="H66" s="5" t="s">
+      <c r="G66" s="5" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2968,11 +2758,8 @@
       <c r="G67" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H67" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2994,11 +2781,8 @@
       <c r="G68" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H68" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3020,11 +2804,8 @@
       <c r="G69" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H69" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -3046,11 +2827,8 @@
       <c r="G70" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H70" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -3072,11 +2850,8 @@
       <c r="G71" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H71" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -3098,11 +2873,8 @@
       <c r="G72" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="H72" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -3121,10 +2893,7 @@
       <c r="F73" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="G73" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="H73" s="5" t="s">
+      <c r="G73" s="5" t="s">
         <v>230</v>
       </c>
     </row>

</xml_diff>